<commit_message>
refactor: update bus identifier to BUS-09 across system, migrations, UI, and exports
</commit_message>
<xml_diff>
--- a/credentials_exports/Boys_Student_Credentials.xlsx
+++ b/credentials_exports/Boys_Student_Credentials.xlsx
@@ -16,7 +16,7 @@
     <t>COLLEGE BUS ATTENDANCE SYSTEM - BOYS CREDENTIALS (21)</t>
   </si>
   <si>
-    <t>Bus: Bus No-09 | Route: College Bus No 09 | Total Records: 21 | Generated: 17/09/2026</t>
+    <t>Bus: BUS-09 | Route: College Bus No 09 | Total Records: 21 | Generated: 17/09/2026</t>
   </si>
   <si>
     <t>S.No</t>
@@ -67,7 +67,7 @@
     <t>student05@college.edu</t>
   </si>
   <si>
-    <t>Bus No-09</t>
+    <t>BUS-09</t>
   </si>
   <si>
     <t>23CS014</t>

</xml_diff>